<commit_message>
Add Priority, Preconditions, Executed By/Date to test cases; Environment, Reported By to bug log
</commit_message>
<xml_diff>
--- a/QA_Documentation/Bug_Report_Log.xlsx
+++ b/QA_Documentation/Bug_Report_Log.xlsx
@@ -476,20 +476,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -540,10 +542,20 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Linked TC ID</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Reported By</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Date Found</t>
         </is>
@@ -598,10 +610,20 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
+          <t>Python 3.11, FastAPI 0.115.0, SQLite, local (uvicorn dev server)</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>TC-02</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Tanisha</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
@@ -655,10 +677,20 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
+          <t>Python 3.11, FastAPI 0.115.0, SQLite, local (uvicorn dev server)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
           <t>TC-04</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Tanisha</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
@@ -716,10 +748,20 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
+          <t>Python 3.11, FastAPI 0.115.0, SQLite, local (uvicorn dev server)</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
           <t>TC-08, TC-10</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Tanisha</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
@@ -774,10 +816,20 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
+          <t>Python 3.11, FastAPI 0.115.0, SQLite, local (uvicorn dev server)</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
           <t>TC-09</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Tanisha</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>
@@ -832,10 +884,20 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
+          <t>Python 3.11, FastAPI 0.115.0, SQLite, local (uvicorn dev server)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
           <t>TC-11</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Tanisha</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>2026-09-23</t>
         </is>

</xml_diff>

<commit_message>
fix: resolve BUG-01 to BUG-05 in approval/leave-request logic; add Bug_Fix_Report.xlsx and update docs to Closed
</commit_message>
<xml_diff>
--- a/QA_Documentation/Bug_Report_Log.xlsx
+++ b/QA_Documentation/Bug_Report_Log.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
         <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -94,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -109,6 +115,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -603,9 +612,9 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -670,9 +679,9 @@
           <t>High</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -741,9 +750,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -809,9 +818,9 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -877,9 +886,9 @@
           <t>Low</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Closed</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">

</xml_diff>